<commit_message>
Commit Done 19-09-2026, 17:39
</commit_message>
<xml_diff>
--- a/src/test/resources/Goldbharath Automation Excel.xlsx
+++ b/src/test/resources/Goldbharath Automation Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/803ce9435f8f2a27/Desktop/Goldbharath Automation Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="11_F25DC773A252ABDACC1048E4595D71765ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF63AEC4-18A9-4546-9B29-723A4358F233}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="11_F25DC773A252ABDACC1048E4595D71765ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3E0823B-E01B-4251-BAC6-B413EA3EB449}"/>
   <bookViews>
-    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="79">
   <si>
     <t>BusinessName</t>
   </si>
@@ -133,13 +133,142 @@
   </si>
   <si>
     <t>Gold Bharath</t>
+  </si>
+  <si>
+    <t>Vikram</t>
+  </si>
+  <si>
+    <t>KYC</t>
+  </si>
+  <si>
+    <t>LLP</t>
+  </si>
+  <si>
+    <t>PROPREITOR</t>
+  </si>
+  <si>
+    <t>PVT LTD</t>
+  </si>
+  <si>
+    <t>LTD</t>
+  </si>
+  <si>
+    <t>Vikram G</t>
+  </si>
+  <si>
+    <t>Propreitor Name</t>
+  </si>
+  <si>
+    <t>CTPPG2544D</t>
+  </si>
+  <si>
+    <t>Pan Number</t>
+  </si>
+  <si>
+    <t>Gst Number</t>
+  </si>
+  <si>
+    <t>36ABCDE1234F1Z5</t>
+  </si>
+  <si>
+    <t>Bank Name</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t>IFSC Code</t>
+  </si>
+  <si>
+    <t>Account Holder Name</t>
+  </si>
+  <si>
+    <t>SBI</t>
+  </si>
+  <si>
+    <t>32809171244</t>
+  </si>
+  <si>
+    <t>SBIN0007457</t>
+  </si>
+  <si>
+    <t>Director Name</t>
+  </si>
+  <si>
+    <t>Director Mobile Number</t>
+  </si>
+  <si>
+    <t>Director Aadhar Number</t>
+  </si>
+  <si>
+    <t>Company GST Number</t>
+  </si>
+  <si>
+    <t>Director CIN Number</t>
+  </si>
+  <si>
+    <t>A/C Number</t>
+  </si>
+  <si>
+    <t>Company Pan Number</t>
+  </si>
+  <si>
+    <t>Company Gst Number</t>
+  </si>
+  <si>
+    <t>436226803420</t>
+  </si>
+  <si>
+    <t>CTPPG2544G</t>
+  </si>
+  <si>
+    <t>Gangavarapu V</t>
+  </si>
+  <si>
+    <t>U51909TG2020PTC123456</t>
+  </si>
+  <si>
+    <t>Director Name(First Director)</t>
+  </si>
+  <si>
+    <t>Director Name(Second Director)</t>
+  </si>
+  <si>
+    <t>32807191243</t>
+  </si>
+  <si>
+    <t>V Gangavarapu</t>
+  </si>
+  <si>
+    <t>Company PAN Number(First Director)</t>
+  </si>
+  <si>
+    <t>Company CIN Number</t>
+  </si>
+  <si>
+    <t>Company Aadhar Number(First Director)</t>
+  </si>
+  <si>
+    <t>Gold And Silver Limits</t>
+  </si>
+  <si>
+    <t>GoldLimit</t>
+  </si>
+  <si>
+    <t>SilverLimit</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>5000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,8 +297,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF3F7F5F"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +341,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -195,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -203,6 +377,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,21 +667,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:L50"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.88671875" customWidth="1"/>
-    <col min="10" max="10" width="43.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.77734375" customWidth="1"/>
+    <col min="11" max="11" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="23.4">
       <c r="E1" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -509,7 +696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -517,7 +704,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -525,7 +712,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -533,7 +720,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -541,7 +728,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -550,7 +737,7 @@
       </c>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -559,116 +746,417 @@
       </c>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="B11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="B13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="B14" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="B15" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="B16" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8">
       <c r="B17" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8">
       <c r="B18" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8">
       <c r="B19" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8">
       <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8">
       <c r="B21" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8">
       <c r="B22" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8">
       <c r="B23" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8">
       <c r="B24" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8">
       <c r="B25" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8">
       <c r="B26" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8">
       <c r="B27" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8">
       <c r="B28" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8">
       <c r="B29" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8">
       <c r="B30" s="2" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8">
+      <c r="C31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="H31" s="7"/>
+    </row>
+    <row r="32" spans="2:8" ht="28.8">
+      <c r="G32" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" s="6" customFormat="1">
+      <c r="B33" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12">
+      <c r="B35" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" t="s">
+        <v>36</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="I35" t="s">
+        <v>36</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="L35" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12">
+      <c r="B36" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" t="s">
+        <v>56</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12">
+      <c r="B37" t="s">
+        <v>46</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12">
+      <c r="B38" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" t="s">
+        <v>61</v>
+      </c>
+      <c r="F38" t="s">
+        <v>64</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I38" t="s">
+        <v>64</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="L38" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12">
+      <c r="B39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E39" t="s">
+        <v>62</v>
+      </c>
+      <c r="F39" t="s">
+        <v>47</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I39" t="s">
+        <v>65</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="L39" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12">
+      <c r="B40" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F40" t="s">
+        <v>66</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I40" t="s">
+        <v>47</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12">
+      <c r="B41" t="s">
+        <v>51</v>
+      </c>
+      <c r="C41" t="s">
+        <v>36</v>
+      </c>
+      <c r="E41" t="s">
+        <v>48</v>
+      </c>
+      <c r="F41" t="s">
+        <v>52</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I41" t="s">
+        <v>66</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="L41" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12">
+      <c r="E42" t="s">
+        <v>60</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H42" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I42" t="s">
+        <v>52</v>
+      </c>
+      <c r="K42" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="L42" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12">
+      <c r="E43" t="s">
+        <v>50</v>
+      </c>
+      <c r="F43" t="s">
+        <v>54</v>
+      </c>
+      <c r="H43" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K43" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12">
+      <c r="E44" t="s">
+        <v>51</v>
+      </c>
+      <c r="F44" t="s">
+        <v>36</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I44" t="s">
+        <v>54</v>
+      </c>
+      <c r="K44" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="L44" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12">
+      <c r="H45" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K45" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="L45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="48" spans="2:12">
+      <c r="E48" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>75</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>